<commit_message>
chore: update job listings and refresh market research data across multiple CSV and JSON files
</commit_message>
<xml_diff>
--- a/Web3_Jobs_Research_Master.xlsx
+++ b/Web3_Jobs_Research_Master.xlsx
@@ -607,22 +607,22 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Growth Lead, Consumer Fraud Reporting</t>
+          <t>Business Development Executive, Public Sector (Europe)</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/trm-labs/73b2f6bd-7f59-4378-8b9f-b0921489c8ef</t>
+          <t>https://jobs.ashbyhq.com/trm-labs/fa2669bc-c77f-42a3-bae5-2c71d16ecca5</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -637,27 +637,27 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Iftother</t>
+          <t>Impossiblecloud</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Head of Business Development - Logos</t>
+          <t>Sales Development Representative (Cloud Services)</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Remote (Worldwide)</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/iftother/jobs/8152733</t>
+          <t>https://jobs.lever.co/impossiblecloud/93b2b790-f749-4aa8-9896-813643c2edc9</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -672,27 +672,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Impossiblecloud</t>
+          <t>Gauntlet</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Inside Sales Manager  - Cloud Services</t>
+          <t>Business Development, US</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>New York City / San Francisco / Los Angeles / Remote</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/impossiblecloud/046c0e1d-afba-4dec-9c85-515b4a1ca15b</t>
+          <t>https://jobs.lever.co/gauntlet/cb1aba05-e9fb-4294-8c2f-865fbeaf04e9</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -707,27 +707,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Orderlynetwork</t>
+          <t>Blockchain</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Associate, Ecosystem Growth &amp; BD</t>
+          <t>Affiliate &amp; Growth Networks Specialist</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/orderly/jobs/4570542008</t>
+          <t>https://job-boards.greenhouse.io/blockchain/jobs/8083268</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -742,27 +742,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Gauntlet</t>
+          <t>Bitgo</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Business Development, APAC</t>
+          <t>Business Development Representative - MENA (Cyprus or Israel)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Singapore / Hong Kong</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/gauntlet/494b0acc-7cfa-4a58-b5dc-c3c914f5d394</t>
+          <t>https://job-boards.greenhouse.io/bitgo/jobs/8534706002</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -855,32 +855,32 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Circle</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Customer Success Manager</t>
+          <t>Principal Product Manager, TradFi</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://ripple.com/careers/all-jobs/job/8141304/?gh_jid=8141304</t>
+          <t>https://careers.circle.com/us/en/job/JR100881/Principal-Product-Manager-TradFi</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Direct company job board link.</t>
+          <t>Pre-scraped job from database.</t>
         </is>
       </c>
     </row>
@@ -890,32 +890,33 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Circle</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Renewals Manager, EMEA</t>
+          <t>VP Of Ecosystem Growth, Pakistan</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>undefined:
+Pakistan</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://ripple.com/careers/all-jobs/job/8179167/?gh_jid=8179167</t>
+          <t>https://careers.circle.com/us/en/job/JR101031/VP-of-Ecosystem-Growth-Pakistan</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Direct company job board link.</t>
+          <t>Pre-scraped job from database.</t>
         </is>
       </c>
     </row>
@@ -925,32 +926,32 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Circle</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Senior Manager, Marketing Analytics</t>
+          <t>Distinguished Software Engineer</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>New York, NY, United States</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://ripple.com/careers/all-jobs/job/7972221/?gh_jid=7972221</t>
+          <t>https://careers.circle.com/us/en/job/JR100849/Distinguished-Software-Engineer</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Direct company job board link.</t>
+          <t>Pre-scraped job from database.</t>
         </is>
       </c>
     </row>
@@ -960,32 +961,32 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Circle</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Senior Manager, Software Engineering – Identity Platform</t>
+          <t>Senior Staff Data Engineer</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://ripple.com/careers/all-jobs/job/8030741/?gh_jid=8030741</t>
+          <t>https://careers.circle.com/us/en/job/JR101020/Senior-Staff-Data-Engineer</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>Direct company job board link.</t>
+          <t>Pre-scraped job from database.</t>
         </is>
       </c>
     </row>
@@ -995,32 +996,32 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Circle</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Senior Manager, Software Engineering – Payments Orchestration</t>
+          <t>VP, Global Head Of Product Security And Risk</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>San Francisco, CA, United States</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://ripple.com/careers/all-jobs/job/7786549/?gh_jid=7786549</t>
+          <t>https://careers.circle.com/us/en/job/JR100878/VP-Global-Head-of-Product-Security-and-Risk</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Direct company job board link.</t>
+          <t>Pre-scraped job from database.</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1102,48 +1103,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Bybit</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Senior P2P Risk Strategy Analyst</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Abu Dhabi, UAE; Kuala Lumpur, Malaysia</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>https://job-boards.eu.greenhouse.io/bybit/jobs/4856962101</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1217,27 +1180,27 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Coinbase</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Customer Success Manager</t>
+          <t>SAM Compliance Lead Analyst</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>London, UK</t>
+          <t>Hybrid - Luxembourg</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://ripple.com/careers/all-jobs/job/8141304/?gh_jid=8141304</t>
+          <t>https://www.coinbase.com/careers/positions/8052192?gh_jid=8052192</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -1252,32 +1215,32 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Coinbase</t>
+          <t>Circle</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Engineering Manager, Market Data &amp; Analytics</t>
+          <t>Principal Product Manager, TradFi</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://www.coinbase.com/careers/positions/8179214?gh_jid=8179214</t>
+          <t>https://careers.circle.com/us/en/job/JR100881/Principal-Product-Manager-TradFi</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Direct company job board link.</t>
+          <t>Pre-scraped job from database.</t>
         </is>
       </c>
     </row>
@@ -1292,22 +1255,22 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Counsel - Regulatory (UK)</t>
+          <t xml:space="preserve">Marketing Manager, CRM Operations </t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/kraken.com/da8b1179-9caa-464c-8eee-395132814f91</t>
+          <t>https://jobs.ashbyhq.com/kraken.com/3bd70487-d97d-47f1-b6f7-7700c17b3bd4</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -1322,27 +1285,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Fireblocks</t>
+          <t>Trmlabs</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Senior Accountant</t>
+          <t>Business Development Executive, Public Sector (Europe)</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Tel Aviv-Yafo, Tel Aviv District, Israel</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://www.fireblocks.com/careers/position?gh_jid=4711456006</t>
+          <t>https://jobs.ashbyhq.com/trm-labs/fa2669bc-c77f-42a3-bae5-2c71d16ecca5</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -1357,27 +1320,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Trmlabs</t>
+          <t>Impossiblecloud</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Growth Lead, Consumer Fraud Reporting</t>
+          <t>Sales Development Representative (Cloud Services)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/trm-labs/73b2f6bd-7f59-4378-8b9f-b0921489c8ef</t>
+          <t>https://jobs.lever.co/impossiblecloud/93b2b790-f749-4aa8-9896-813643c2edc9</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -1407,7 +1370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1464,84 +1427,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Coinbase</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Engineering Manager, Market Data &amp; Analytics</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Remote - USA</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>https://www.coinbase.com/careers/positions/8179214?gh_jid=8179214</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Subzero labs</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/subzero/f36ca76a-4fca-4ba4-8a67-c4946d6072db</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1552,7 +1441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1609,48 +1498,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Fiber</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Business Analytics Strategic Partnerships Tokenisation Manager</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>https://web3.career/business-analytics-strategic-partnerships-tokenisation-manager-binance/153663</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2008,27 +1859,27 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Trmlabs</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Senior International Sales Recruiter, UK/EMEA</t>
+          <t>HR Business Partner</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/trm-labs/b6994b6a-0b46-4311-b0f6-3b71d9b5ded9</t>
+          <t>https://jobs.lever.co/binance/d3bd1209-bce1-45af-80dc-17d03159c019</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -2048,7 +1899,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Pioneer Talent Program - Applied Data Scientist</t>
+          <t>Pioneer Talent Program - Research Data Scientist</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -2058,12 +1909,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/binance/9d5af64f-be8d-4cbf-a096-5a5a4294afbe</t>
+          <t>https://jobs.lever.co/binance/efa6ff12-8332-4e08-b587-e88f7ea68177</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -2078,27 +1929,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Whitebit</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Talent Programs Manager</t>
+          <t>Senior Talent Acquisition Operations Specialist (Contract)</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://whitebit.hurma.work/public-vacancies/1261</t>
+          <t>https://jobs.lever.co/binance/f5e9f843-fa64-40c8-af06-1f1a58943897</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -2113,27 +1964,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Digital asset</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Global Talent Acquisition Coordinator</t>
+          <t>Senior Talent Acquisition Specialist (Technical and Product)</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/digitalassetcorp/jobs/4392277009</t>
+          <t>https://jobs.lever.co/binance/a1124a16-3dfe-4547-b0e9-90aa402ebfde</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -2148,32 +1999,32 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Dragonflycapital</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>People Ops - Dragonfly Portfolio</t>
+          <t>Talent Acquisition Specialist</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>New York City • Hybrid</t>
+          <t>UAE, Dubai</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.gem.com/dragonfly-careers/4621670004</t>
+          <t>https://jobs.lever.co/binance/89670300-3ec1-438d-b7b4-ff59441c03af</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Pre-scraped job from database.</t>
+          <t>Direct company job board link.</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2117,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Senior Market Data Engineer</t>
+          <t>Senior Software Engineer, Data Layer</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -2276,12 +2127,12 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://www.coinbase.com/careers/positions/8180833?gh_jid=8180833</t>
+          <t>https://www.coinbase.com/careers/positions/8064873?gh_jid=8064873</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -2301,7 +2152,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Senior Network Engineer</t>
+          <t>Senior Software Engineer - Frontend - Coinbase Card team</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -2311,12 +2162,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://www.coinbase.com/careers/positions/8179311?gh_jid=8179311</t>
+          <t>https://www.coinbase.com/careers/positions/8088201?gh_jid=8088201</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -2336,22 +2187,22 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Consumer</t>
+          <t>Senior Software Engineer, Simple Trade Experience</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Remote - Singapore</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://www.coinbase.com/careers/positions/8067033?gh_jid=8067033</t>
+          <t>https://www.coinbase.com/careers/positions/8103569?gh_jid=8103569</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -2371,22 +2222,22 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Core Reliability</t>
+          <t>Senior Software Engineer, Stablecoins</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Remote - Canada</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://www.coinbase.com/careers/positions/8097944?gh_jid=8097944</t>
+          <t>https://www.coinbase.com/careers/positions/8104873?gh_jid=8104873</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -2406,22 +2257,22 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Data Engineering Platform</t>
+          <t>Senior Software Engineer - Trading</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Remote - USA</t>
+          <t>Remote - Singapore</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://www.coinbase.com/careers/positions/8082199?gh_jid=8082199</t>
+          <t>https://www.coinbase.com/careers/positions/7866674?gh_jid=7866674</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -2514,27 +2365,27 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Kraken</t>
+          <t>Bitpanda</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Platform Product Manager — Payward Services</t>
+          <t>Senior Product Manager – Securities &amp; Commodities</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Vienna, Vienna, Austria</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/kraken.com/c6298ed5-978b-49ea-8cec-ce90f275d540</t>
+          <t>https://job-boards.eu.greenhouse.io/bitpanda/jobs/4954725101</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -2549,27 +2400,27 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Moonpay</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Product Manager, Identity</t>
+          <t>Senior Product Manager - Exchange, Trading</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>London - Hybrid</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/moonpay/d9e4fd9d-5b4e-4ba1-b637-a21f9eec54b4</t>
+          <t>https://jobs.lever.co/crypto/fbb256a2-46a3-41b7-942d-5ba87018c0dc</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -2584,27 +2435,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Bitpanda</t>
+          <t>Bastion</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Senior Product Manager - Growth, Engagement &amp; Retention</t>
+          <t>Product Manager</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Vienna, Vienna, Austria</t>
+          <t>US Remote</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.eu.greenhouse.io/bitpanda/jobs/4959025101</t>
+          <t>https://jobs.ashbyhq.com/Bastion/04a403af-fcae-4e10-9960-b9970243a4aa</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -2624,22 +2475,22 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Principal Product Manager, Affiliate &amp; KOL - Onshore Markets</t>
+          <t>Principal Product Manager, Growth</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Hong Kong, Hong Kong SAR; Singapore, Singapore</t>
+          <t>San Jose, California, United States</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/okx/jobs/7777902003</t>
+          <t>https://job-boards.greenhouse.io/okx/jobs/7713617003</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -2654,27 +2505,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Moonpay</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Senior Product Manager, KYB - MoonPay Enterprise</t>
+          <t>Senior Product Manager - Predictions, OG</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>London - Hybrid</t>
+          <t>San Francisco</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/moonpay/91e69ea7-bfc1-4b8a-bbc5-8439bacfcb57</t>
+          <t>https://jobs.lever.co/crypto/f6a19e4d-1150-476a-8566-ea0e7f2fd96a</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -2772,7 +2623,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Senior Product Designer, Defi</t>
+          <t>Senior Product Designer, Wallets</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -2782,12 +2633,12 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/okx/jobs/7747651003</t>
+          <t>https://job-boards.greenhouse.io/okx/jobs/7985087003</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -2802,27 +2653,27 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Product Designer - Predictions, OG</t>
+          <t>Creative Ops Lead</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/crypto/629ce48a-c8ed-4b22-bf29-5b516241e3f9</t>
+          <t>https://jobs.ashbyhq.com/polymarket/031c38a6-3c76-4440-8569-b070c744d9a9</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -2837,27 +2688,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Sports Design Lead</t>
+          <t>Binance Accelerator Program - Graphic Design (MENA)</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>UAE, Dubai</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/polymarket/3a42a698-7569-4eb8-9bec-9214c7b51692</t>
+          <t>https://jobs.lever.co/binance/3785f1c4-3d3a-494a-9d0b-51e68f84ac08</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -2872,27 +2723,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Stellar</t>
+          <t>Alpaca</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Brand Designer</t>
+          <t>Senior Graphic Designer</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Remote - North America</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/stellar/72644c96-916c-4644-aff3-3382fc4eb0ff</t>
+          <t>https://job-boards.greenhouse.io/alpaca/jobs/5744207004</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -2907,27 +2758,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Symbiotic.fi</t>
+          <t>Asterdex</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Senior Product Designer</t>
+          <t>Creative Designer</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>APAC</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/Symbiotic/ffc40ecb-169d-4027-bd5b-326e5710b897</t>
+          <t>https://jobs.lever.co/pioneer-services/d9ad7005-3b50-44de-ba62-d4ce48c3c907</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -3096,7 +2947,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr. Systems Analyst, Finance, Enterprise Apps </t>
+          <t>Strategic Finance Manager, Platform</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -3106,12 +2957,12 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://www.coinbase.com/careers/positions/8154856?gh_jid=8154856</t>
+          <t>https://www.coinbase.com/careers/positions/8148248?gh_jid=8148248</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -3126,27 +2977,27 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Fireblocks</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Senior Accountant</t>
+          <t>Assistant Financial Controller</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Tel Aviv-Yafo, Tel Aviv District, Israel</t>
+          <t>Chicago,IL</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://www.fireblocks.com/careers/position?gh_jid=4711456006</t>
+          <t>https://jobs.lever.co/crypto/bf231bb5-1c89-481a-b856-29771cdf5656</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -3166,22 +3017,22 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Senior Finance Analyst </t>
+          <t>Senior Finance Manager - Group Consolidation</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Sliema, Malta</t>
+          <t>Singapore, Singapore</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/okx/jobs/7805828003</t>
+          <t>https://job-boards.greenhouse.io/okx/jobs/7802200003</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -3196,27 +3047,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Animocabrands</t>
+          <t>Solanafoundation</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Senior Associate, Accounting</t>
+          <t>Senior Accountant, Financial Operations</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Hong Kong</t>
+          <t>Remote-International</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/animocabrands/bb994ec6-4017-47ea-8291-224a7358566f</t>
+          <t>https://jobs.ashbyhq.com/Solana%20Foundation/e9a5aba3-4b4d-4635-b26a-57b7d4591dfd</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -3231,27 +3082,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Xapo</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Treasury Manager (Remote - Work from Anywhere)</t>
+          <t>Assistant Manager, Financial and Management Reporting</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Gibraltar - Remote</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/xapo61/jobs/7812568003</t>
+          <t>https://jobs.lever.co/crypto/b8182b66-c109-4a81-a091-ca00ccd7201c</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -3281,7 +3132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3344,65 +3195,30 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Bitpanda</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Fraud Operations Manager</t>
+          <t xml:space="preserve">Associate, Customer Support - Live chat </t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Vienna, Vienna, Austria</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/polymarket/6703b7cd-2b97-4bed-9445-3ab8d74150f0</t>
+          <t>https://job-boards.eu.greenhouse.io/bitpanda/jobs/4969789101</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>Customer Success Manager/Lead</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>San Francisco or Boulder</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/foundation/e209bb72-3d83-4f74-b8de-6f44773bde6f</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>Direct company job board link.</t>
         </is>
@@ -3414,7 +3230,6 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3489,27 +3304,27 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Merchandising Operations Manager - Surface,  OG</t>
+          <t>Binance Accelerator Program - Product Operations (Earn &amp; TradFi)</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>San Francisco</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/crypto/ed7f015a-45b0-4072-9bfc-27345a4e8db8</t>
+          <t>https://jobs.lever.co/binance/77d4c5cf-a604-454f-9e35-79d5ce32c318</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -3524,27 +3339,27 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Trust-wallet</t>
+          <t>Alpaca</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Operations Lead</t>
+          <t>Crypto Operations Associate - APAC</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Remote - Global</t>
+          <t xml:space="preserve">Remote - Anywhere </t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/trust-wallet/044e897e-1f08-42a2-b6b9-9272e60622f4</t>
+          <t>https://job-boards.greenhouse.io/alpaca/jobs/4431262004</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -3559,27 +3374,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Alpaca</t>
+          <t>Hyperbolic</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Brokerage Operations Manager - Saudi </t>
+          <t>GTM (Operations)</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Remote - EMEA</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/alpaca/jobs/5857441004</t>
+          <t>https://jobs.ashbyhq.com/hyperbolic/51206c65-0350-4b22-8340-e86f70debb70</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -3599,22 +3414,22 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Binance Accelerator Program - Operations (Web3)</t>
+          <t>Operational Risk / Enterprise Risk Management Framework (ERMF) Specialist</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Hong Kong</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/binance/ff9b1c8a-b0de-4bb4-a81e-d2cd51f57e31</t>
+          <t>https://jobs.lever.co/binance/744cb1d2-2f53-4819-8b5f-ef82a4460776</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -3629,27 +3444,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Alpaca</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Corporate Operations Lead  </t>
+          <t>Operations Analyst - Brazil</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Remote - North America  and Remote  - EMEA</t>
+          <t>Brazil, Sao Paulo</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/alpaca/jobs/6172681004</t>
+          <t>https://jobs.lever.co/binance/1b148889-f898-4579-84f7-dbccfa5fee4a</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -3679,7 +3494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3736,48 +3551,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Foundation</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Software Engineering</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>San Francisco, Boulder, or Austin</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/foundation/2fffc9a2-7e3a-461c-8bb1-675540024014</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3851,27 +3628,27 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Okx</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Lifecycle Director</t>
+          <t>Workplace IT Specialist</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>New York, United States</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/polymarket/0fe656ba-7e91-466e-ab7a-f719f7f96a1c</t>
+          <t>https://job-boards.greenhouse.io/okx/jobs/7808492003</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -3886,12 +3663,12 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Chainalysis</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Deal Desk Manager (Fixed-Term)</t>
+          <t>Senior Data Scientist / Analyst, Institutional</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -3901,12 +3678,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/chainalysis-careers/8d8570f8-17b6-446a-9a3c-c65d5484da63</t>
+          <t>https://jobs.ashbyhq.com/polymarket/4bcdc897-3126-4d8e-ba8a-d398255cad6e</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -3921,12 +3698,12 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Chainalysis</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Senior Payment Risk Analyst</t>
+          <t>Senior People Systems &amp; Integrations Analyst</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -3936,12 +3713,12 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/polymarket/62e81b7f-d045-495b-9f36-0c91392870f3</t>
+          <t>https://jobs.ashbyhq.com/chainalysis-careers/f28e555e-ba54-4ea5-a41b-4c534438d019</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -3956,27 +3733,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Meshpay</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Senior Data Scientist / Analyst, Product</t>
+          <t>Head of Forward Deployed Engineering</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>New York, NY</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/polymarket/ddcc0048-6175-4c9b-847a-ce02e4508377</t>
+          <t>https://job-boards.greenhouse.io/mesh/jobs/5380179008</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -3991,27 +3768,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Rwa.xyz</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Product Lead, Data Licensing</t>
+          <t>Senior Research Analyst</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/polymarket/f7ece09b-5045-421e-8d7f-1d1b88fd97d8</t>
+          <t>https://jobs.ashbyhq.com/RWA.xyz/b3b035a7-3067-4639-998b-863476b22ae3</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -4041,7 +3818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4098,48 +3875,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Blockchain</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Business Lead</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>London</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>https://job-boards.greenhouse.io/blockchain/jobs/8045350</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4150,7 +3889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4207,84 +3946,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Tangem</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Web Attribution Analyst</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Remote / Zug, Switzerland</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>https://careers.tangem.com/web-attribution-analyst</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Tangem</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>UX Writer</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>Remote / Zug, Switzerland</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>https://careers.tangem.com/ux-writer</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4363,7 +4028,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Senior Enterprise Product  Marketing Manager, Base</t>
+          <t>Senior Internal Communications Manager, People</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -4373,12 +4038,12 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://www.coinbase.com/careers/positions/8084049?gh_jid=8084049</t>
+          <t>https://www.coinbase.com/careers/positions/8162914?gh_jid=8162914</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -4393,12 +4058,12 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Kraken</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Social Media Manager/ Content Creator</t>
+          <t xml:space="preserve">Marketing Manager, CRM Operations </t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -4408,12 +4073,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/crypto/ff3dc7ba-662e-4e49-82c2-e6143bb93712</t>
+          <t>https://jobs.ashbyhq.com/kraken.com/3bd70487-d97d-47f1-b6f7-7700c17b3bd4</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -4428,27 +4093,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Polymarket</t>
+          <t>Coinmarketcap</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Polymarket 2026 Summer Internship — Marketing &amp; Finance</t>
+          <t>Senior Marketing Specialist</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/polymarket/9fbf8f68-5f92-434d-a00b-c79f99f5a10e</t>
+          <t>https://jobs.lever.co/coinmarketcap/b71b07d0-5a27-4101-b30d-ea442a2e096f</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -4463,27 +4128,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Rain</t>
+          <t>Polymarket</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Product Marketing Manager - Money Movement</t>
+          <t>Performance Marketing Lead, International</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>New York, NY</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/rain/6aa4cf9f-58bd-45a5-bce0-e0da60ee7a8a</t>
+          <t>https://jobs.ashbyhq.com/polymarket/e6fc54f3-339e-4196-a221-53e8d7c2049f</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -4498,27 +4163,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Coinmarketcap</t>
+          <t>Windranger</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Global VP Marketing/CMO</t>
+          <t>Mantle Squad US – Marketing &amp; Growth</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>New York</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/coinmarketcap/3badc309-fe0c-41f6-8e78-5236dc331b8c</t>
+          <t>https://jobs.ashbyhq.com/windranger/83df91bb-55ba-4f01-b586-659f2c2c5172</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -4690,7 +4355,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4747,48 +4412,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Sahara ai</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Community Manager</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Seoul</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>https://jobs.ashbyhq.com/sahara/ba33f05b-0858-4b5e-92cf-630852b624f1</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>06 Sep 2026</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Direct company job board link.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4938,7 +4565,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Backend Engineer, Agent Tools</t>
+          <t>Staff Data Engineer - AI Platform</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -4948,12 +4575,12 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/trm-labs/1eff4d33-7cf1-4682-a548-dcc4abd913f3</t>
+          <t>https://jobs.ashbyhq.com/trm-labs/74fc12c1-be22-496e-812d-1316276c91e8</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -4968,27 +4595,27 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Impossiblecloud</t>
+          <t>Okx</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Product Manager / Director – GPU &amp; AI Services</t>
+          <t>AI Agent Security Research Engineer</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>APAC; Hong Kong, Hong Kong SAR; Singapore, Singapore</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/impossiblecloud/78255efa-0423-4cf3-9bd8-8229e150616b</t>
+          <t>https://job-boards.greenhouse.io/okx/jobs/7650023003</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -5003,27 +4630,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Moonpay</t>
+          <t>Trmlabs</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Staff Machine Learning Engineer</t>
+          <t>Data Platform Engineer - AI Platform</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>London - Hybrid</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/moonpay/a12369da-ded2-4798-b176-b22928e9cf21</t>
+          <t>https://jobs.ashbyhq.com/trm-labs/2a784630-702d-4b49-a033-5cbd0d9c8a94</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -5038,27 +4665,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Okx</t>
+          <t>Trmlabs</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">AI Agent Product Expert (Middleware) </t>
+          <t>Senior Data Platform Engineer - AI Platform</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Hong Kong, Hong Kong SAR</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/okx/jobs/7731745003</t>
+          <t>https://jobs.ashbyhq.com/trm-labs/cf1c3e90-d709-4a64-825f-7c0f0768965a</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -5078,7 +4705,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Senior Data Engineer - AI Platform</t>
+          <t>Staff Data Platform Engineer - AI Platform</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -5088,12 +4715,12 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/trm-labs/45e886bf-748d-41cb-9748-258440d12b61</t>
+          <t>https://jobs.ashbyhq.com/trm-labs/a1ed36fb-8be9-40a9-8452-5641996130c3</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -5123,7 +4750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5180,10 +4807,48 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Treasury Asset Management</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/binance/c3d1aa01-9df6-4778-953f-9320b995a791</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>08 Sep 2026</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Direct company job board link.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5265,7 +4930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5322,10 +4987,48 @@
         </is>
       </c>
     </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Bitpanda</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Intern, CEO Office</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Vienna, Vienna, Austria</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>https://job-boards.eu.greenhouse.io/bitpanda/jobs/4959756101</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>08 Sep 2026</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Direct company job board link.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5404,22 +5107,22 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Senior Derivatives Trader</t>
+          <t>Trading Operations Team Lead</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Cayman Islands</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/anchorage/c2b42959-0a4b-4e85-9901-8a875d586902</t>
+          <t>https://jobs.lever.co/anchorage/b3c332bc-ffc5-4a2f-ab3e-de136d326408</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -5439,22 +5142,22 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Senior Algorithmic Trader / Liquidity Researcher</t>
+          <t>Senior Data Analyst, Trading</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Taiwan, Taipei</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/binance/08a7954d-65ed-4c3c-9de6-266fb4cbddbc</t>
+          <t>https://jobs.lever.co/binance/e92d8b5f-0f0a-4569-884f-4f45c8ad024c</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -5469,32 +5172,32 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Kappa lab</t>
+          <t>Freedx</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Quant Trader</t>
+          <t>Senior Trading Behavior &amp; Flow Risk Analyst</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>London, United Kingdom (Hybrid)</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.gohire.io/kappa-lab-ltd-8jxmdnnt/quant-trader-297472/?ref=aHR0cHM6Ly9hcHAuZ29oaXJlLmlvLw==</t>
+          <t>https://apply.workable.com/freedx/j/53837BBE09/</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Direct company job board link.</t>
+          <t>Pre-scraped job from database.</t>
         </is>
       </c>
     </row>
@@ -5504,27 +5207,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Freedx</t>
+          <t>Robinhood</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Business Analyst (Middle / Senior) - Trading Team (CEX)</t>
+          <t>Customer Experience Representative, Active Trader</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Remote</t>
+          <t>Chicago, IL; Denver, CO; Westlake, TX</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/freedx/j/2F76FAD2AA/</t>
+          <t>https://boards.greenhouse.io/robinhood/jobs/8011599?gh_src=NaN&amp;gh_jid=8011599</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -5539,27 +5242,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Crypto-finance</t>
+          <t>Freedx</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Application Manager - Trading</t>
+          <t>Python Trading Research Analyst</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>On-site</t>
+          <t>Remote</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/crypto-finance/j/B2ADF0BD4D/</t>
+          <t>https://apply.workable.com/freedx/j/C5153916B3/</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -5652,27 +5355,27 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Gate.io</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>区块链开发工程师</t>
+          <t>Binance Accelerator Program - Research Data Scientist</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>APAC-C1</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/gate/4f2aa64b-2252-4c57-8e70-a34f7c71cf63</t>
+          <t>https://jobs.lever.co/binance/ca44ee4e-392b-4745-9ad9-8e287f5a6d37</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -5692,7 +5395,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Binance Accelerator Program - Applied Data Scientist</t>
+          <t>Binance Accelerator Program - Research On Chain Data Analyst</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -5702,12 +5405,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/binance/ae1a07c1-c971-403c-906b-79d8c16e4f2d</t>
+          <t>https://jobs.lever.co/binance/fb9d588a-e49e-4496-a464-9c6c5cc4ca46</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -5722,27 +5425,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Gate.io</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>测试负责人</t>
+          <t>Business Analytics &amp; Strategic Partnerships (Tokenisation) Manager</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>APAC-C1</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/gate/0505a0c2-d2e9-47f5-8400-a7e184b72555</t>
+          <t>https://jobs.lever.co/binance/281f252b-ad90-45e1-b8f2-eca5e8c1a8e9</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -5757,27 +5460,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Gate.io</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>社交产品负责人</t>
+          <t>Business Intelligence/ Data Analystics</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>APAC-C1</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/gate/41166281-1fb5-40fd-bd61-a1467d2c0418</t>
+          <t>https://jobs.lever.co/binance/e2cec219-a165-4baa-bb22-33be2e2f3063</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -5797,22 +5500,22 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Binance Accelerator Program - QA</t>
+          <t>Chief Information Security Officer (Korea)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>South Korea, Seoul</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/binance/2603f3c0-75cb-4d49-b8de-cb4ade0e8b39</t>
+          <t>https://jobs.lever.co/binance/0400c0b4-c07e-42c5-a000-205995dcd8ef</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
@@ -5981,22 +5684,22 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Risk Manager - Country &amp; Operational Risk</t>
+          <t>SAM Compliance Lead Analyst</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>Remote - UK</t>
+          <t>Hybrid - Luxembourg</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>https://www.coinbase.com/careers/positions/7774051?gh_jid=7774051</t>
+          <t>https://www.coinbase.com/careers/positions/8052192?gh_jid=8052192</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -6016,7 +5719,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Counsel - Regulatory (UK)</t>
+          <t>Internal Audit Financial Crime &amp; Conduct Manager</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -6026,12 +5729,12 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/kraken.com/da8b1179-9caa-464c-8eee-395132814f91</t>
+          <t>https://jobs.ashbyhq.com/kraken.com/042f0568-49a6-4c25-b7a2-c578844b1e2f</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -6046,27 +5749,27 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Impossiblecloud</t>
+          <t>Blockchain</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Legal Intern</t>
+          <t xml:space="preserve">Compliance Analytics Associate </t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Buenos Aires</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/impossiblecloud/fdb042c2-56ae-42b7-82c4-898bc628818f</t>
+          <t>https://job-boards.greenhouse.io/blockchain/jobs/8155035</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -6081,27 +5784,27 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Moonpay</t>
+          <t>Bitgo</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Product Counsel</t>
+          <t>Associate General Counsel</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>New York - Hybrid</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/moonpay/eb7aeddb-a021-4ab5-9dfc-e74ec143b8de</t>
+          <t>https://job-boards.greenhouse.io/bitgo/jobs/8627534002</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
@@ -6116,27 +5819,27 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Gauntlet</t>
+          <t>Coinbase</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Head of Compliance</t>
+          <t>Senior Analyst, Compliance Technology</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>New York City / San Francisco / Los Angeles / Remote</t>
+          <t>Remote - USA</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.lever.co/gauntlet/64f960f1-3ed2-4ad5-aa7c-6e71a3c60aca</t>
+          <t>https://www.coinbase.com/careers/positions/8067443?gh_jid=8067443</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>06 Sep 2026</t>
+          <t>08 Sep 2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">

</xml_diff>